<commit_message>
Auto update RUP 2026-07-14 08:00:38
</commit_message>
<xml_diff>
--- a/output/rup/2026/Rekap RUP Tahun 2026 (2026-07-14).xlsx
+++ b/output/rup/2026/Rekap RUP Tahun 2026 (2026-07-14).xlsx
@@ -523,10 +523,10 @@
         <v>1581202807</v>
       </c>
       <c r="D2" s="3" t="n">
-        <v>0</v>
+        <v>67</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>0</v>
+        <v>486896807</v>
       </c>
       <c r="F2" s="3" t="n">
         <v>4</v>
@@ -535,16 +535,16 @@
         <v>1094306000</v>
       </c>
       <c r="H2" s="3" t="n">
-        <v>4</v>
+        <v>71</v>
       </c>
       <c r="I2" s="3" t="n">
-        <v>1094306000</v>
+        <v>1581202807</v>
       </c>
       <c r="J2" s="3" t="n">
-        <v>-486896807</v>
+        <v>0</v>
       </c>
       <c r="K2" s="4" t="n">
-        <v>69.20718804415834</v>
+        <v>100</v>
       </c>
     </row>
     <row r="3">
@@ -560,10 +560,10 @@
         <v>830740630</v>
       </c>
       <c r="D3" s="3" t="n">
-        <v>0</v>
+        <v>77</v>
       </c>
       <c r="E3" s="3" t="n">
-        <v>0</v>
+        <v>830740630</v>
       </c>
       <c r="F3" s="3" t="n">
         <v>0</v>
@@ -572,16 +572,16 @@
         <v>0</v>
       </c>
       <c r="H3" s="3" t="n">
-        <v>0</v>
+        <v>77</v>
       </c>
       <c r="I3" s="3" t="n">
-        <v>0</v>
+        <v>830740630</v>
       </c>
       <c r="J3" s="3" t="n">
-        <v>-830740630</v>
+        <v>0</v>
       </c>
       <c r="K3" s="4" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="4">
@@ -597,10 +597,10 @@
         <v>1385846979</v>
       </c>
       <c r="D4" s="3" t="n">
-        <v>0</v>
+        <v>98</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>0</v>
+        <v>1385846979</v>
       </c>
       <c r="F4" s="3" t="n">
         <v>0</v>
@@ -609,16 +609,16 @@
         <v>0</v>
       </c>
       <c r="H4" s="3" t="n">
-        <v>0</v>
+        <v>98</v>
       </c>
       <c r="I4" s="3" t="n">
-        <v>0</v>
+        <v>1385846979</v>
       </c>
       <c r="J4" s="3" t="n">
-        <v>-1385846979</v>
+        <v>0</v>
       </c>
       <c r="K4" s="4" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="5">
@@ -634,10 +634,10 @@
         <v>1363592000</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>0</v>
+        <v>101</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>0</v>
+        <v>1363592000</v>
       </c>
       <c r="F5" s="3" t="n">
         <v>0</v>
@@ -646,16 +646,16 @@
         <v>0</v>
       </c>
       <c r="H5" s="3" t="n">
-        <v>0</v>
+        <v>101</v>
       </c>
       <c r="I5" s="3" t="n">
-        <v>0</v>
+        <v>1363592000</v>
       </c>
       <c r="J5" s="3" t="n">
-        <v>-1363592000</v>
+        <v>0</v>
       </c>
       <c r="K5" s="4" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="6">
@@ -671,10 +671,10 @@
         <v>3636937261</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>0</v>
+        <v>79</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>0</v>
+        <v>2417247421</v>
       </c>
       <c r="F6" s="3" t="n">
         <v>5</v>
@@ -683,16 +683,16 @@
         <v>1219689840</v>
       </c>
       <c r="H6" s="3" t="n">
-        <v>5</v>
+        <v>84</v>
       </c>
       <c r="I6" s="3" t="n">
-        <v>1219689840</v>
+        <v>3636937261</v>
       </c>
       <c r="J6" s="3" t="n">
-        <v>-2417247421</v>
+        <v>0</v>
       </c>
       <c r="K6" s="4" t="n">
-        <v>33.53618037569991</v>
+        <v>100</v>
       </c>
     </row>
     <row r="7">
@@ -708,10 +708,10 @@
         <v>1145858598</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>0</v>
+        <v>127</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>0</v>
+        <v>1145858598</v>
       </c>
       <c r="F7" s="3" t="n">
         <v>0</v>
@@ -720,16 +720,16 @@
         <v>0</v>
       </c>
       <c r="H7" s="3" t="n">
-        <v>0</v>
+        <v>127</v>
       </c>
       <c r="I7" s="3" t="n">
-        <v>0</v>
+        <v>1145858598</v>
       </c>
       <c r="J7" s="3" t="n">
-        <v>-1145858598</v>
+        <v>0</v>
       </c>
       <c r="K7" s="4" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="8">
@@ -819,10 +819,10 @@
         <v>2454000424</v>
       </c>
       <c r="D10" s="3" t="n">
-        <v>0</v>
+        <v>91</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>0</v>
+        <v>2454000424</v>
       </c>
       <c r="F10" s="3" t="n">
         <v>0</v>
@@ -831,16 +831,16 @@
         <v>0</v>
       </c>
       <c r="H10" s="3" t="n">
-        <v>0</v>
+        <v>91</v>
       </c>
       <c r="I10" s="3" t="n">
-        <v>0</v>
+        <v>2454000424</v>
       </c>
       <c r="J10" s="3" t="n">
-        <v>-2454000424</v>
+        <v>0</v>
       </c>
       <c r="K10" s="4" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="11">
@@ -856,10 +856,10 @@
         <v>978184643</v>
       </c>
       <c r="D11" s="3" t="n">
-        <v>0</v>
+        <v>81</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>0</v>
+        <v>978184643</v>
       </c>
       <c r="F11" s="3" t="n">
         <v>0</v>
@@ -868,16 +868,16 @@
         <v>0</v>
       </c>
       <c r="H11" s="3" t="n">
-        <v>0</v>
+        <v>81</v>
       </c>
       <c r="I11" s="3" t="n">
-        <v>0</v>
+        <v>978184643</v>
       </c>
       <c r="J11" s="3" t="n">
-        <v>-978184643</v>
+        <v>0</v>
       </c>
       <c r="K11" s="4" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="12">
@@ -893,10 +893,10 @@
         <v>4891035773</v>
       </c>
       <c r="D12" s="3" t="n">
-        <v>0</v>
+        <v>114</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>0</v>
+        <v>4891035773</v>
       </c>
       <c r="F12" s="3" t="n">
         <v>0</v>
@@ -905,16 +905,16 @@
         <v>0</v>
       </c>
       <c r="H12" s="3" t="n">
-        <v>0</v>
+        <v>114</v>
       </c>
       <c r="I12" s="3" t="n">
-        <v>0</v>
+        <v>4891035773</v>
       </c>
       <c r="J12" s="3" t="n">
-        <v>-4891035773</v>
+        <v>0</v>
       </c>
       <c r="K12" s="4" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="13">
@@ -930,10 +930,10 @@
         <v>4363300381</v>
       </c>
       <c r="D13" s="3" t="n">
-        <v>0</v>
+        <v>58</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>0</v>
+        <v>4363300381</v>
       </c>
       <c r="F13" s="3" t="n">
         <v>0</v>
@@ -942,16 +942,16 @@
         <v>0</v>
       </c>
       <c r="H13" s="3" t="n">
-        <v>0</v>
+        <v>58</v>
       </c>
       <c r="I13" s="3" t="n">
-        <v>0</v>
+        <v>4363300381</v>
       </c>
       <c r="J13" s="3" t="n">
-        <v>-4363300381</v>
+        <v>0</v>
       </c>
       <c r="K13" s="4" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="14">
@@ -967,10 +967,10 @@
         <v>15288269163</v>
       </c>
       <c r="D14" s="3" t="n">
-        <v>0</v>
+        <v>149</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>0</v>
+        <v>15288269163</v>
       </c>
       <c r="F14" s="3" t="n">
         <v>0</v>
@@ -979,16 +979,16 @@
         <v>0</v>
       </c>
       <c r="H14" s="3" t="n">
-        <v>0</v>
+        <v>149</v>
       </c>
       <c r="I14" s="3" t="n">
-        <v>0</v>
+        <v>15288269163</v>
       </c>
       <c r="J14" s="3" t="n">
-        <v>-15288269163</v>
+        <v>0</v>
       </c>
       <c r="K14" s="4" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="15">
@@ -1004,10 +1004,10 @@
         <v>2474291200</v>
       </c>
       <c r="D15" s="3" t="n">
-        <v>0</v>
+        <v>109</v>
       </c>
       <c r="E15" s="3" t="n">
-        <v>0</v>
+        <v>2474291200</v>
       </c>
       <c r="F15" s="3" t="n">
         <v>0</v>
@@ -1016,16 +1016,16 @@
         <v>0</v>
       </c>
       <c r="H15" s="3" t="n">
-        <v>0</v>
+        <v>109</v>
       </c>
       <c r="I15" s="3" t="n">
-        <v>0</v>
+        <v>2474291200</v>
       </c>
       <c r="J15" s="3" t="n">
-        <v>-2474291200</v>
+        <v>0</v>
       </c>
       <c r="K15" s="4" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="16">
@@ -1041,10 +1041,10 @@
         <v>105032048100</v>
       </c>
       <c r="D16" s="3" t="n">
-        <v>0</v>
+        <v>385</v>
       </c>
       <c r="E16" s="3" t="n">
-        <v>0</v>
+        <v>104997048100</v>
       </c>
       <c r="F16" s="3" t="n">
         <v>1</v>
@@ -1053,16 +1053,16 @@
         <v>35000000</v>
       </c>
       <c r="H16" s="3" t="n">
-        <v>1</v>
+        <v>386</v>
       </c>
       <c r="I16" s="3" t="n">
-        <v>35000000</v>
+        <v>105032048100</v>
       </c>
       <c r="J16" s="3" t="n">
-        <v>-104997048100</v>
+        <v>0</v>
       </c>
       <c r="K16" s="4" t="n">
-        <v>0.0333231624376941</v>
+        <v>100</v>
       </c>
     </row>
     <row r="17">
@@ -1078,10 +1078,10 @@
         <v>2187676345</v>
       </c>
       <c r="D17" s="3" t="n">
-        <v>0</v>
+        <v>66</v>
       </c>
       <c r="E17" s="3" t="n">
-        <v>0</v>
+        <v>2187676345</v>
       </c>
       <c r="F17" s="3" t="n">
         <v>0</v>
@@ -1090,16 +1090,16 @@
         <v>0</v>
       </c>
       <c r="H17" s="3" t="n">
-        <v>0</v>
+        <v>66</v>
       </c>
       <c r="I17" s="3" t="n">
-        <v>0</v>
+        <v>2187676345</v>
       </c>
       <c r="J17" s="3" t="n">
-        <v>-2187676345</v>
+        <v>0</v>
       </c>
       <c r="K17" s="4" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="18">
@@ -1115,10 +1115,10 @@
         <v>1662695697</v>
       </c>
       <c r="D18" s="3" t="n">
-        <v>0</v>
+        <v>66</v>
       </c>
       <c r="E18" s="3" t="n">
-        <v>0</v>
+        <v>1662695697</v>
       </c>
       <c r="F18" s="3" t="n">
         <v>0</v>
@@ -1127,16 +1127,16 @@
         <v>0</v>
       </c>
       <c r="H18" s="3" t="n">
-        <v>0</v>
+        <v>66</v>
       </c>
       <c r="I18" s="3" t="n">
-        <v>0</v>
+        <v>1662695697</v>
       </c>
       <c r="J18" s="3" t="n">
-        <v>-1662695697</v>
+        <v>0</v>
       </c>
       <c r="K18" s="4" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="19">
@@ -1152,10 +1152,10 @@
         <v>2181147677</v>
       </c>
       <c r="D19" s="3" t="n">
-        <v>0</v>
+        <v>129</v>
       </c>
       <c r="E19" s="3" t="n">
-        <v>0</v>
+        <v>2181147677</v>
       </c>
       <c r="F19" s="3" t="n">
         <v>0</v>
@@ -1164,16 +1164,16 @@
         <v>0</v>
       </c>
       <c r="H19" s="3" t="n">
-        <v>0</v>
+        <v>129</v>
       </c>
       <c r="I19" s="3" t="n">
-        <v>0</v>
+        <v>2181147677</v>
       </c>
       <c r="J19" s="3" t="n">
-        <v>-2181147677</v>
+        <v>0</v>
       </c>
       <c r="K19" s="4" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="20">
@@ -1189,10 +1189,10 @@
         <v>575172642</v>
       </c>
       <c r="D20" s="3" t="n">
-        <v>0</v>
+        <v>33</v>
       </c>
       <c r="E20" s="3" t="n">
-        <v>0</v>
+        <v>575172642</v>
       </c>
       <c r="F20" s="3" t="n">
         <v>0</v>
@@ -1201,16 +1201,16 @@
         <v>0</v>
       </c>
       <c r="H20" s="3" t="n">
-        <v>0</v>
+        <v>33</v>
       </c>
       <c r="I20" s="3" t="n">
-        <v>0</v>
+        <v>575172642</v>
       </c>
       <c r="J20" s="3" t="n">
-        <v>-575172642</v>
+        <v>0</v>
       </c>
       <c r="K20" s="4" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="21">
@@ -1226,10 +1226,10 @@
         <v>61655471600</v>
       </c>
       <c r="D21" s="3" t="n">
-        <v>0</v>
+        <v>274</v>
       </c>
       <c r="E21" s="3" t="n">
-        <v>0</v>
+        <v>9467977800</v>
       </c>
       <c r="F21" s="3" t="n">
         <v>30</v>
@@ -1238,16 +1238,16 @@
         <v>52187493800</v>
       </c>
       <c r="H21" s="3" t="n">
-        <v>30</v>
+        <v>304</v>
       </c>
       <c r="I21" s="3" t="n">
-        <v>52187493800</v>
+        <v>61655471600</v>
       </c>
       <c r="J21" s="3" t="n">
-        <v>-9467977800</v>
+        <v>0</v>
       </c>
       <c r="K21" s="4" t="n">
-        <v>84.64373468517918</v>
+        <v>100</v>
       </c>
     </row>
     <row r="22">
@@ -1263,10 +1263,10 @@
         <v>10654182000</v>
       </c>
       <c r="D22" s="3" t="n">
-        <v>0</v>
+        <v>75</v>
       </c>
       <c r="E22" s="3" t="n">
-        <v>0</v>
+        <v>10500724500</v>
       </c>
       <c r="F22" s="3" t="n">
         <v>0</v>
@@ -1275,16 +1275,16 @@
         <v>0</v>
       </c>
       <c r="H22" s="3" t="n">
-        <v>0</v>
+        <v>75</v>
       </c>
       <c r="I22" s="3" t="n">
-        <v>0</v>
+        <v>10500724500</v>
       </c>
       <c r="J22" s="3" t="n">
-        <v>-10654182000</v>
+        <v>-153457500</v>
       </c>
       <c r="K22" s="4" t="n">
-        <v>0</v>
+        <v>98.55965009796154</v>
       </c>
     </row>
     <row r="23">
@@ -1300,10 +1300,10 @@
         <v>8063419229</v>
       </c>
       <c r="D23" s="3" t="n">
-        <v>0</v>
+        <v>130</v>
       </c>
       <c r="E23" s="3" t="n">
-        <v>0</v>
+        <v>8063419229</v>
       </c>
       <c r="F23" s="3" t="n">
         <v>0</v>
@@ -1312,16 +1312,16 @@
         <v>0</v>
       </c>
       <c r="H23" s="3" t="n">
-        <v>0</v>
+        <v>130</v>
       </c>
       <c r="I23" s="3" t="n">
-        <v>0</v>
+        <v>8063419229</v>
       </c>
       <c r="J23" s="3" t="n">
-        <v>-8063419229</v>
+        <v>0</v>
       </c>
       <c r="K23" s="4" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="24">
@@ -1337,10 +1337,10 @@
         <v>11668621099</v>
       </c>
       <c r="D24" s="3" t="n">
-        <v>0</v>
+        <v>130</v>
       </c>
       <c r="E24" s="3" t="n">
-        <v>0</v>
+        <v>11668621099</v>
       </c>
       <c r="F24" s="3" t="n">
         <v>0</v>
@@ -1349,16 +1349,16 @@
         <v>0</v>
       </c>
       <c r="H24" s="3" t="n">
-        <v>0</v>
+        <v>130</v>
       </c>
       <c r="I24" s="3" t="n">
-        <v>0</v>
+        <v>11668621099</v>
       </c>
       <c r="J24" s="3" t="n">
-        <v>-11668621099</v>
+        <v>0</v>
       </c>
       <c r="K24" s="4" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="25">
@@ -1374,10 +1374,10 @@
         <v>532966503</v>
       </c>
       <c r="D25" s="3" t="n">
-        <v>0</v>
+        <v>81</v>
       </c>
       <c r="E25" s="3" t="n">
-        <v>0</v>
+        <v>532966503</v>
       </c>
       <c r="F25" s="3" t="n">
         <v>0</v>
@@ -1386,16 +1386,16 @@
         <v>0</v>
       </c>
       <c r="H25" s="3" t="n">
-        <v>0</v>
+        <v>81</v>
       </c>
       <c r="I25" s="3" t="n">
-        <v>0</v>
+        <v>532966503</v>
       </c>
       <c r="J25" s="3" t="n">
-        <v>-532966503</v>
+        <v>0</v>
       </c>
       <c r="K25" s="4" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="26">
@@ -1411,10 +1411,10 @@
         <v>12076302500</v>
       </c>
       <c r="D26" s="3" t="n">
-        <v>0</v>
+        <v>164</v>
       </c>
       <c r="E26" s="3" t="n">
-        <v>0</v>
+        <v>11831302500</v>
       </c>
       <c r="F26" s="3" t="n">
         <v>1</v>
@@ -1423,16 +1423,16 @@
         <v>245000000</v>
       </c>
       <c r="H26" s="3" t="n">
-        <v>1</v>
+        <v>165</v>
       </c>
       <c r="I26" s="3" t="n">
-        <v>245000000</v>
+        <v>12076302500</v>
       </c>
       <c r="J26" s="3" t="n">
-        <v>-11831302500</v>
+        <v>0</v>
       </c>
       <c r="K26" s="4" t="n">
-        <v>2.028766669268181</v>
+        <v>100</v>
       </c>
     </row>
     <row r="27">
@@ -1448,10 +1448,10 @@
         <v>28552934680</v>
       </c>
       <c r="D27" s="3" t="n">
-        <v>0</v>
+        <v>280</v>
       </c>
       <c r="E27" s="3" t="n">
-        <v>0</v>
+        <v>28552934680</v>
       </c>
       <c r="F27" s="3" t="n">
         <v>0</v>
@@ -1460,16 +1460,16 @@
         <v>0</v>
       </c>
       <c r="H27" s="3" t="n">
-        <v>0</v>
+        <v>280</v>
       </c>
       <c r="I27" s="3" t="n">
-        <v>0</v>
+        <v>28552934680</v>
       </c>
       <c r="J27" s="3" t="n">
-        <v>-28552934680</v>
+        <v>0</v>
       </c>
       <c r="K27" s="4" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="28">
@@ -1485,10 +1485,10 @@
         <v>1858317230</v>
       </c>
       <c r="D28" s="3" t="n">
-        <v>0</v>
+        <v>109</v>
       </c>
       <c r="E28" s="3" t="n">
-        <v>0</v>
+        <v>1858317230</v>
       </c>
       <c r="F28" s="3" t="n">
         <v>0</v>
@@ -1497,16 +1497,16 @@
         <v>0</v>
       </c>
       <c r="H28" s="3" t="n">
-        <v>0</v>
+        <v>109</v>
       </c>
       <c r="I28" s="3" t="n">
-        <v>0</v>
+        <v>1858317230</v>
       </c>
       <c r="J28" s="3" t="n">
-        <v>-1858317230</v>
+        <v>0</v>
       </c>
       <c r="K28" s="4" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="29">
@@ -1522,10 +1522,10 @@
         <v>1417613763</v>
       </c>
       <c r="D29" s="3" t="n">
-        <v>0</v>
+        <v>89</v>
       </c>
       <c r="E29" s="3" t="n">
-        <v>0</v>
+        <v>1417613763</v>
       </c>
       <c r="F29" s="3" t="n">
         <v>0</v>
@@ -1534,16 +1534,16 @@
         <v>0</v>
       </c>
       <c r="H29" s="3" t="n">
-        <v>0</v>
+        <v>89</v>
       </c>
       <c r="I29" s="3" t="n">
-        <v>0</v>
+        <v>1417613763</v>
       </c>
       <c r="J29" s="3" t="n">
-        <v>-1417613763</v>
+        <v>0</v>
       </c>
       <c r="K29" s="4" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="30">
@@ -1559,10 +1559,10 @@
         <v>1292926000</v>
       </c>
       <c r="D30" s="3" t="n">
-        <v>0</v>
+        <v>55</v>
       </c>
       <c r="E30" s="3" t="n">
-        <v>0</v>
+        <v>1292926000</v>
       </c>
       <c r="F30" s="3" t="n">
         <v>0</v>
@@ -1571,16 +1571,16 @@
         <v>0</v>
       </c>
       <c r="H30" s="3" t="n">
-        <v>0</v>
+        <v>55</v>
       </c>
       <c r="I30" s="3" t="n">
-        <v>0</v>
+        <v>1292926000</v>
       </c>
       <c r="J30" s="3" t="n">
-        <v>-1292926000</v>
+        <v>0</v>
       </c>
       <c r="K30" s="4" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="31">
@@ -1596,10 +1596,10 @@
         <v>5257374241</v>
       </c>
       <c r="D31" s="3" t="n">
-        <v>0</v>
+        <v>34</v>
       </c>
       <c r="E31" s="3" t="n">
-        <v>0</v>
+        <v>5051110241</v>
       </c>
       <c r="F31" s="3" t="n">
         <v>0</v>
@@ -1608,16 +1608,16 @@
         <v>0</v>
       </c>
       <c r="H31" s="3" t="n">
-        <v>0</v>
+        <v>34</v>
       </c>
       <c r="I31" s="3" t="n">
-        <v>0</v>
+        <v>5051110241</v>
       </c>
       <c r="J31" s="3" t="n">
-        <v>-5257374241</v>
+        <v>-206264000</v>
       </c>
       <c r="K31" s="4" t="n">
-        <v>0</v>
+        <v>96.07667267832227</v>
       </c>
     </row>
     <row r="32">
@@ -1633,10 +1633,10 @@
         <v>4701405808</v>
       </c>
       <c r="D32" s="3" t="n">
-        <v>0</v>
+        <v>184</v>
       </c>
       <c r="E32" s="3" t="n">
-        <v>0</v>
+        <v>4606645808</v>
       </c>
       <c r="F32" s="3" t="n">
         <v>2</v>
@@ -1645,16 +1645,16 @@
         <v>94760000</v>
       </c>
       <c r="H32" s="3" t="n">
-        <v>2</v>
+        <v>186</v>
       </c>
       <c r="I32" s="3" t="n">
-        <v>94760000</v>
+        <v>4701405808</v>
       </c>
       <c r="J32" s="3" t="n">
-        <v>-4606645808</v>
+        <v>0</v>
       </c>
       <c r="K32" s="4" t="n">
-        <v>2.015567340278404</v>
+        <v>100</v>
       </c>
     </row>
     <row r="33">
@@ -1670,10 +1670,10 @@
         <v>465249566</v>
       </c>
       <c r="D33" s="3" t="n">
-        <v>0</v>
+        <v>66</v>
       </c>
       <c r="E33" s="3" t="n">
-        <v>0</v>
+        <v>465249566</v>
       </c>
       <c r="F33" s="3" t="n">
         <v>0</v>
@@ -1682,16 +1682,16 @@
         <v>0</v>
       </c>
       <c r="H33" s="3" t="n">
-        <v>0</v>
+        <v>66</v>
       </c>
       <c r="I33" s="3" t="n">
-        <v>0</v>
+        <v>465249566</v>
       </c>
       <c r="J33" s="3" t="n">
-        <v>-465249566</v>
+        <v>0</v>
       </c>
       <c r="K33" s="4" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="34">
@@ -1707,10 +1707,10 @@
         <v>948269958</v>
       </c>
       <c r="D34" s="3" t="n">
-        <v>0</v>
+        <v>49</v>
       </c>
       <c r="E34" s="3" t="n">
-        <v>0</v>
+        <v>507369966</v>
       </c>
       <c r="F34" s="3" t="n">
         <v>1</v>
@@ -1719,16 +1719,16 @@
         <v>440899992</v>
       </c>
       <c r="H34" s="3" t="n">
-        <v>1</v>
+        <v>50</v>
       </c>
       <c r="I34" s="3" t="n">
-        <v>440899992</v>
+        <v>948269958</v>
       </c>
       <c r="J34" s="3" t="n">
-        <v>-507369966</v>
+        <v>0</v>
       </c>
       <c r="K34" s="4" t="n">
-        <v>46.49519773144601</v>
+        <v>100</v>
       </c>
     </row>
     <row r="35">
@@ -1744,10 +1744,10 @@
         <v>943247000</v>
       </c>
       <c r="D35" s="3" t="n">
-        <v>0</v>
+        <v>111</v>
       </c>
       <c r="E35" s="3" t="n">
-        <v>0</v>
+        <v>774999698</v>
       </c>
       <c r="F35" s="3" t="n">
         <v>5</v>
@@ -1756,16 +1756,16 @@
         <v>168247302</v>
       </c>
       <c r="H35" s="3" t="n">
-        <v>5</v>
+        <v>116</v>
       </c>
       <c r="I35" s="3" t="n">
-        <v>168247302</v>
+        <v>943247000</v>
       </c>
       <c r="J35" s="3" t="n">
-        <v>-774999698</v>
+        <v>0</v>
       </c>
       <c r="K35" s="4" t="n">
-        <v>17.83703547427132</v>
+        <v>100</v>
       </c>
     </row>
     <row r="36">
@@ -1781,10 +1781,10 @@
         <v>312595476</v>
       </c>
       <c r="D36" s="3" t="n">
-        <v>0</v>
+        <v>59</v>
       </c>
       <c r="E36" s="3" t="n">
-        <v>0</v>
+        <v>312595476</v>
       </c>
       <c r="F36" s="3" t="n">
         <v>0</v>
@@ -1793,16 +1793,16 @@
         <v>0</v>
       </c>
       <c r="H36" s="3" t="n">
-        <v>0</v>
+        <v>59</v>
       </c>
       <c r="I36" s="3" t="n">
-        <v>0</v>
+        <v>312595476</v>
       </c>
       <c r="J36" s="3" t="n">
-        <v>-312595476</v>
+        <v>0</v>
       </c>
       <c r="K36" s="4" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="37">
@@ -1818,10 +1818,10 @@
         <v>219851775</v>
       </c>
       <c r="D37" s="3" t="n">
-        <v>0</v>
+        <v>38</v>
       </c>
       <c r="E37" s="3" t="n">
-        <v>0</v>
+        <v>219851775</v>
       </c>
       <c r="F37" s="3" t="n">
         <v>0</v>
@@ -1830,16 +1830,16 @@
         <v>0</v>
       </c>
       <c r="H37" s="3" t="n">
-        <v>0</v>
+        <v>38</v>
       </c>
       <c r="I37" s="3" t="n">
-        <v>0</v>
+        <v>219851775</v>
       </c>
       <c r="J37" s="3" t="n">
-        <v>-219851775</v>
+        <v>0</v>
       </c>
       <c r="K37" s="4" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="38">
@@ -2373,10 +2373,10 @@
         <v>2405886712</v>
       </c>
       <c r="D52" s="3" t="n">
-        <v>0</v>
+        <v>22</v>
       </c>
       <c r="E52" s="3" t="n">
-        <v>0</v>
+        <v>2374286712</v>
       </c>
       <c r="F52" s="3" t="n">
         <v>3</v>
@@ -2385,16 +2385,16 @@
         <v>31600000</v>
       </c>
       <c r="H52" s="3" t="n">
-        <v>3</v>
+        <v>25</v>
       </c>
       <c r="I52" s="3" t="n">
-        <v>31600000</v>
+        <v>2405886712</v>
       </c>
       <c r="J52" s="3" t="n">
-        <v>-2374286712</v>
+        <v>0</v>
       </c>
       <c r="K52" s="4" t="n">
-        <v>1.313445053018772</v>
+        <v>100</v>
       </c>
     </row>
     <row r="53">
@@ -2558,10 +2558,10 @@
         <v>1801912000</v>
       </c>
       <c r="D57" s="3" t="n">
-        <v>0</v>
+        <v>56</v>
       </c>
       <c r="E57" s="3" t="n">
-        <v>0</v>
+        <v>1780912000</v>
       </c>
       <c r="F57" s="3" t="n">
         <v>1</v>
@@ -2570,16 +2570,16 @@
         <v>21000000</v>
       </c>
       <c r="H57" s="3" t="n">
-        <v>1</v>
+        <v>57</v>
       </c>
       <c r="I57" s="3" t="n">
-        <v>21000000</v>
+        <v>1801912000</v>
       </c>
       <c r="J57" s="3" t="n">
-        <v>-1780912000</v>
+        <v>0</v>
       </c>
       <c r="K57" s="4" t="n">
-        <v>1.165428722379339</v>
+        <v>100</v>
       </c>
     </row>
     <row r="58">
@@ -2595,10 +2595,10 @@
         <v>1367075285</v>
       </c>
       <c r="D58" s="3" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="E58" s="3" t="n">
-        <v>0</v>
+        <v>721339185</v>
       </c>
       <c r="F58" s="3" t="n">
         <v>0</v>
@@ -2607,16 +2607,16 @@
         <v>0</v>
       </c>
       <c r="H58" s="3" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="I58" s="3" t="n">
-        <v>0</v>
+        <v>721339185</v>
       </c>
       <c r="J58" s="3" t="n">
-        <v>-1367075285</v>
+        <v>-645736100</v>
       </c>
       <c r="K58" s="4" t="n">
-        <v>0</v>
+        <v>52.76513977794573</v>
       </c>
     </row>
     <row r="59">
@@ -2632,10 +2632,10 @@
         <v>338454320</v>
       </c>
       <c r="D59" s="3" t="n">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="E59" s="3" t="n">
-        <v>0</v>
+        <v>338454320</v>
       </c>
       <c r="F59" s="3" t="n">
         <v>0</v>
@@ -2644,16 +2644,16 @@
         <v>0</v>
       </c>
       <c r="H59" s="3" t="n">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="I59" s="3" t="n">
-        <v>0</v>
+        <v>338454320</v>
       </c>
       <c r="J59" s="3" t="n">
-        <v>-338454320</v>
+        <v>0</v>
       </c>
       <c r="K59" s="4" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="60">
@@ -2669,10 +2669,10 @@
         <v>887410440</v>
       </c>
       <c r="D60" s="3" t="n">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="E60" s="3" t="n">
-        <v>0</v>
+        <v>887410440</v>
       </c>
       <c r="F60" s="3" t="n">
         <v>0</v>
@@ -2681,16 +2681,16 @@
         <v>0</v>
       </c>
       <c r="H60" s="3" t="n">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="I60" s="3" t="n">
-        <v>0</v>
+        <v>887410440</v>
       </c>
       <c r="J60" s="3" t="n">
-        <v>-887410440</v>
+        <v>0</v>
       </c>
       <c r="K60" s="4" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="61">
@@ -2706,10 +2706,10 @@
         <v>1424797850</v>
       </c>
       <c r="D61" s="3" t="n">
-        <v>0</v>
+        <v>21</v>
       </c>
       <c r="E61" s="3" t="n">
-        <v>0</v>
+        <v>212772837</v>
       </c>
       <c r="F61" s="3" t="n">
         <v>0</v>
@@ -2718,16 +2718,16 @@
         <v>0</v>
       </c>
       <c r="H61" s="3" t="n">
-        <v>0</v>
+        <v>21</v>
       </c>
       <c r="I61" s="3" t="n">
-        <v>0</v>
+        <v>212772837</v>
       </c>
       <c r="J61" s="3" t="n">
-        <v>-1424797850</v>
+        <v>-1212025013</v>
       </c>
       <c r="K61" s="4" t="n">
-        <v>0</v>
+        <v>14.93354562543732</v>
       </c>
     </row>
     <row r="62">
@@ -2743,10 +2743,10 @@
         <v>1117262389</v>
       </c>
       <c r="D62" s="3" t="n">
-        <v>0</v>
+        <v>42</v>
       </c>
       <c r="E62" s="3" t="n">
-        <v>0</v>
+        <v>1116362329</v>
       </c>
       <c r="F62" s="3" t="n">
         <v>0</v>
@@ -2755,16 +2755,16 @@
         <v>0</v>
       </c>
       <c r="H62" s="3" t="n">
-        <v>0</v>
+        <v>42</v>
       </c>
       <c r="I62" s="3" t="n">
-        <v>0</v>
+        <v>1116362329</v>
       </c>
       <c r="J62" s="3" t="n">
-        <v>-1117262389</v>
+        <v>-900060</v>
       </c>
       <c r="K62" s="4" t="n">
-        <v>0</v>
+        <v>99.91944058899132</v>
       </c>
     </row>
     <row r="63">
@@ -2780,10 +2780,10 @@
         <v>509262312</v>
       </c>
       <c r="D63" s="3" t="n">
-        <v>0</v>
+        <v>43</v>
       </c>
       <c r="E63" s="3" t="n">
-        <v>0</v>
+        <v>509262312</v>
       </c>
       <c r="F63" s="3" t="n">
         <v>0</v>
@@ -2792,16 +2792,16 @@
         <v>0</v>
       </c>
       <c r="H63" s="3" t="n">
-        <v>0</v>
+        <v>43</v>
       </c>
       <c r="I63" s="3" t="n">
-        <v>0</v>
+        <v>509262312</v>
       </c>
       <c r="J63" s="3" t="n">
-        <v>-509262312</v>
+        <v>0</v>
       </c>
       <c r="K63" s="4" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="64">
@@ -2817,10 +2817,10 @@
         <v>373421530</v>
       </c>
       <c r="D64" s="3" t="n">
-        <v>0</v>
+        <v>17</v>
       </c>
       <c r="E64" s="3" t="n">
-        <v>0</v>
+        <v>373421530</v>
       </c>
       <c r="F64" s="3" t="n">
         <v>0</v>
@@ -2829,16 +2829,16 @@
         <v>0</v>
       </c>
       <c r="H64" s="3" t="n">
-        <v>0</v>
+        <v>17</v>
       </c>
       <c r="I64" s="3" t="n">
-        <v>0</v>
+        <v>373421530</v>
       </c>
       <c r="J64" s="3" t="n">
-        <v>-373421530</v>
+        <v>0</v>
       </c>
       <c r="K64" s="4" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="65">
@@ -2854,10 +2854,10 @@
         <v>552591787</v>
       </c>
       <c r="D65" s="3" t="n">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="E65" s="3" t="n">
-        <v>0</v>
+        <v>552591787</v>
       </c>
       <c r="F65" s="3" t="n">
         <v>0</v>
@@ -2866,16 +2866,16 @@
         <v>0</v>
       </c>
       <c r="H65" s="3" t="n">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="I65" s="3" t="n">
-        <v>0</v>
+        <v>552591787</v>
       </c>
       <c r="J65" s="3" t="n">
-        <v>-552591787</v>
+        <v>0</v>
       </c>
       <c r="K65" s="4" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="66">
@@ -2891,10 +2891,10 @@
         <v>735655752</v>
       </c>
       <c r="D66" s="3" t="n">
-        <v>0</v>
+        <v>38</v>
       </c>
       <c r="E66" s="3" t="n">
-        <v>0</v>
+        <v>541055752</v>
       </c>
       <c r="F66" s="3" t="n">
         <v>1</v>
@@ -2903,16 +2903,16 @@
         <v>194600000</v>
       </c>
       <c r="H66" s="3" t="n">
-        <v>1</v>
+        <v>39</v>
       </c>
       <c r="I66" s="3" t="n">
-        <v>194600000</v>
+        <v>735655752</v>
       </c>
       <c r="J66" s="3" t="n">
-        <v>-541055752</v>
+        <v>0</v>
       </c>
       <c r="K66" s="4" t="n">
-        <v>26.45259001522767</v>
+        <v>100</v>
       </c>
     </row>
     <row r="67">
@@ -2928,10 +2928,10 @@
         <v>289499767</v>
       </c>
       <c r="D67" s="3" t="n">
-        <v>0</v>
+        <v>22</v>
       </c>
       <c r="E67" s="3" t="n">
-        <v>0</v>
+        <v>289499767</v>
       </c>
       <c r="F67" s="3" t="n">
         <v>0</v>
@@ -2940,16 +2940,16 @@
         <v>0</v>
       </c>
       <c r="H67" s="3" t="n">
-        <v>0</v>
+        <v>22</v>
       </c>
       <c r="I67" s="3" t="n">
-        <v>0</v>
+        <v>289499767</v>
       </c>
       <c r="J67" s="3" t="n">
-        <v>-289499767</v>
+        <v>0</v>
       </c>
       <c r="K67" s="4" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="68">
@@ -2965,10 +2965,10 @@
         <v>429267455</v>
       </c>
       <c r="D68" s="3" t="n">
-        <v>0</v>
+        <v>36</v>
       </c>
       <c r="E68" s="3" t="n">
-        <v>0</v>
+        <v>429267455</v>
       </c>
       <c r="F68" s="3" t="n">
         <v>0</v>
@@ -2977,16 +2977,16 @@
         <v>0</v>
       </c>
       <c r="H68" s="3" t="n">
-        <v>0</v>
+        <v>36</v>
       </c>
       <c r="I68" s="3" t="n">
-        <v>0</v>
+        <v>429267455</v>
       </c>
       <c r="J68" s="3" t="n">
-        <v>-429267455</v>
+        <v>0</v>
       </c>
       <c r="K68" s="4" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="69">
@@ -3002,10 +3002,10 @@
         <v>153251633</v>
       </c>
       <c r="D69" s="3" t="n">
-        <v>0</v>
+        <v>26</v>
       </c>
       <c r="E69" s="3" t="n">
-        <v>0</v>
+        <v>153251633</v>
       </c>
       <c r="F69" s="3" t="n">
         <v>0</v>
@@ -3014,16 +3014,16 @@
         <v>0</v>
       </c>
       <c r="H69" s="3" t="n">
-        <v>0</v>
+        <v>26</v>
       </c>
       <c r="I69" s="3" t="n">
-        <v>0</v>
+        <v>153251633</v>
       </c>
       <c r="J69" s="3" t="n">
-        <v>-153251633</v>
+        <v>0</v>
       </c>
       <c r="K69" s="4" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="70">
@@ -3039,10 +3039,10 @@
         <v>329330796</v>
       </c>
       <c r="D70" s="3" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="E70" s="3" t="n">
-        <v>0</v>
+        <v>329330796</v>
       </c>
       <c r="F70" s="3" t="n">
         <v>0</v>
@@ -3051,16 +3051,16 @@
         <v>0</v>
       </c>
       <c r="H70" s="3" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="I70" s="3" t="n">
-        <v>0</v>
+        <v>329330796</v>
       </c>
       <c r="J70" s="3" t="n">
-        <v>-329330796</v>
+        <v>0</v>
       </c>
       <c r="K70" s="4" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="71">
@@ -3076,10 +3076,10 @@
         <v>270659900</v>
       </c>
       <c r="D71" s="3" t="n">
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="E71" s="3" t="n">
-        <v>0</v>
+        <v>270659900</v>
       </c>
       <c r="F71" s="3" t="n">
         <v>0</v>
@@ -3088,16 +3088,16 @@
         <v>0</v>
       </c>
       <c r="H71" s="3" t="n">
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="I71" s="3" t="n">
-        <v>0</v>
+        <v>270659900</v>
       </c>
       <c r="J71" s="3" t="n">
-        <v>-270659900</v>
+        <v>0</v>
       </c>
       <c r="K71" s="4" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="72">
@@ -3113,10 +3113,10 @@
         <v>654395500</v>
       </c>
       <c r="D72" s="3" t="n">
-        <v>0</v>
+        <v>41</v>
       </c>
       <c r="E72" s="3" t="n">
-        <v>0</v>
+        <v>654395500</v>
       </c>
       <c r="F72" s="3" t="n">
         <v>0</v>
@@ -3125,16 +3125,16 @@
         <v>0</v>
       </c>
       <c r="H72" s="3" t="n">
-        <v>0</v>
+        <v>41</v>
       </c>
       <c r="I72" s="3" t="n">
-        <v>0</v>
+        <v>654395500</v>
       </c>
       <c r="J72" s="3" t="n">
-        <v>-654395500</v>
+        <v>0</v>
       </c>
       <c r="K72" s="4" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="73">
@@ -3150,10 +3150,10 @@
         <v>448879549</v>
       </c>
       <c r="D73" s="3" t="n">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="E73" s="3" t="n">
-        <v>0</v>
+        <v>448879549</v>
       </c>
       <c r="F73" s="3" t="n">
         <v>0</v>
@@ -3162,16 +3162,16 @@
         <v>0</v>
       </c>
       <c r="H73" s="3" t="n">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="I73" s="3" t="n">
-        <v>0</v>
+        <v>448879549</v>
       </c>
       <c r="J73" s="3" t="n">
-        <v>-448879549</v>
+        <v>0</v>
       </c>
       <c r="K73" s="4" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="74">
@@ -3187,10 +3187,10 @@
         <v>1291889268</v>
       </c>
       <c r="D74" s="3" t="n">
-        <v>0</v>
+        <v>22</v>
       </c>
       <c r="E74" s="3" t="n">
-        <v>0</v>
+        <v>350390301</v>
       </c>
       <c r="F74" s="3" t="n">
         <v>0</v>
@@ -3199,16 +3199,16 @@
         <v>0</v>
       </c>
       <c r="H74" s="3" t="n">
-        <v>0</v>
+        <v>22</v>
       </c>
       <c r="I74" s="3" t="n">
-        <v>0</v>
+        <v>350390301</v>
       </c>
       <c r="J74" s="3" t="n">
-        <v>-1291889268</v>
+        <v>-941498967</v>
       </c>
       <c r="K74" s="4" t="n">
-        <v>0</v>
+        <v>27.12231687956092</v>
       </c>
     </row>
     <row r="75">
@@ -3261,10 +3261,10 @@
         <v>992988041</v>
       </c>
       <c r="D76" s="3" t="n">
-        <v>0</v>
+        <v>36</v>
       </c>
       <c r="E76" s="3" t="n">
-        <v>0</v>
+        <v>992988041</v>
       </c>
       <c r="F76" s="3" t="n">
         <v>0</v>
@@ -3273,16 +3273,16 @@
         <v>0</v>
       </c>
       <c r="H76" s="3" t="n">
-        <v>0</v>
+        <v>36</v>
       </c>
       <c r="I76" s="3" t="n">
-        <v>0</v>
+        <v>992988041</v>
       </c>
       <c r="J76" s="3" t="n">
-        <v>-992988041</v>
+        <v>0</v>
       </c>
       <c r="K76" s="4" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="77">
@@ -3298,10 +3298,10 @@
         <v>85061928740</v>
       </c>
       <c r="D77" s="3" t="n">
-        <v>0</v>
+        <v>85</v>
       </c>
       <c r="E77" s="3" t="n">
-        <v>0</v>
+        <v>85061928740</v>
       </c>
       <c r="F77" s="3" t="n">
         <v>0</v>
@@ -3310,16 +3310,16 @@
         <v>0</v>
       </c>
       <c r="H77" s="3" t="n">
-        <v>0</v>
+        <v>85</v>
       </c>
       <c r="I77" s="3" t="n">
-        <v>0</v>
+        <v>85061928740</v>
       </c>
       <c r="J77" s="3" t="n">
-        <v>-85061928740</v>
+        <v>0</v>
       </c>
       <c r="K77" s="4" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="78">
@@ -3335,10 +3335,10 @@
         <v>1028700867</v>
       </c>
       <c r="D78" s="3" t="n">
-        <v>0</v>
+        <v>56</v>
       </c>
       <c r="E78" s="3" t="n">
-        <v>0</v>
+        <v>1028700867</v>
       </c>
       <c r="F78" s="3" t="n">
         <v>0</v>
@@ -3347,16 +3347,16 @@
         <v>0</v>
       </c>
       <c r="H78" s="3" t="n">
-        <v>0</v>
+        <v>56</v>
       </c>
       <c r="I78" s="3" t="n">
-        <v>0</v>
+        <v>1028700867</v>
       </c>
       <c r="J78" s="3" t="n">
-        <v>-1028700867</v>
+        <v>0</v>
       </c>
       <c r="K78" s="4" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="79">
@@ -3372,10 +3372,10 @@
         <v>8905641688</v>
       </c>
       <c r="D79" s="3" t="n">
-        <v>0</v>
+        <v>133</v>
       </c>
       <c r="E79" s="3" t="n">
-        <v>0</v>
+        <v>8755641688</v>
       </c>
       <c r="F79" s="3" t="n">
         <v>1</v>
@@ -3384,16 +3384,16 @@
         <v>150000000</v>
       </c>
       <c r="H79" s="3" t="n">
-        <v>1</v>
+        <v>134</v>
       </c>
       <c r="I79" s="3" t="n">
-        <v>150000000</v>
+        <v>8905641688</v>
       </c>
       <c r="J79" s="3" t="n">
-        <v>-8755641688</v>
+        <v>0</v>
       </c>
       <c r="K79" s="4" t="n">
-        <v>1.684325568612524</v>
+        <v>100</v>
       </c>
     </row>
     <row r="80">
@@ -3409,10 +3409,10 @@
         <v>11974816559</v>
       </c>
       <c r="D80" s="3" t="n">
-        <v>0</v>
+        <v>191</v>
       </c>
       <c r="E80" s="3" t="n">
-        <v>0</v>
+        <v>11799027759</v>
       </c>
       <c r="F80" s="3" t="n">
         <v>2</v>
@@ -3421,16 +3421,16 @@
         <v>175788800</v>
       </c>
       <c r="H80" s="3" t="n">
-        <v>2</v>
+        <v>193</v>
       </c>
       <c r="I80" s="3" t="n">
-        <v>175788800</v>
+        <v>11974816559</v>
       </c>
       <c r="J80" s="3" t="n">
-        <v>-11799027759</v>
+        <v>0</v>
       </c>
       <c r="K80" s="4" t="n">
-        <v>1.467987414536894</v>
+        <v>100</v>
       </c>
     </row>
     <row r="81">

</xml_diff>